<commit_message>
progress: 7 village workbooks (sivaramans-llin 2026-10-08T18:00:59Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Periyapuliyur_13.389385_80.036223.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Periyapuliyur_13.389385_80.036223.xlsx
@@ -1514,6 +1514,11 @@
           <t>2</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1B, 2, 3A, 3B</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1521,6 +1526,11 @@
           <t>20</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1528,6 +1538,11 @@
           <t>21</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16A, 16B, 2, 3A, 3B, 3C, 3D, 3E, 3F, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1535,6 +1550,11 @@
           <t>22</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 2, 3, 4, 5, 6, 7A, 7B, 7C, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1542,11 +1562,21 @@
           <t>23</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
           <t>24</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1, 10, 2A, 2B, 2C, 2D, 3, 4, 5, 6, 7, 8, 9</t>
         </is>
       </c>
     </row>

</xml_diff>